<commit_message>
feat(per-subject): enumerate legal subjects per incident (pelaku/PSE/konsumen/regulator)
Stage 1 of the per-subject (subjek hukum) redesign addressing the conflation bias:
a single incident binds multiple legal subjects with different positions and
regimes. Each incident now carries subjek_hukum[] = {peran, pihak, posisi_hukum,
objek_hukum, dasar_hukum} templated by offence category, bilingual. Consumer party
is distinguished from the robbed institution in fraud cases. Surfaced on incident
cards as a 'Subjek Hukum' block (role-coloured); removed redundant single
Pelaku/PSE rows.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/network/Vallidation.xlsx
+++ b/data/network/Vallidation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/solehhasanwahid/Library/CloudStorage/GoogleDrive-wahid@uinponorogo.ac.id/Drive Saya/BAHAN PENELITIAN/JESSD/DIGITAL AI GOVERNANCE/data/network/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B0F91B8-F27A-524B-8B66-B7D9085F8038}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37EF608C-A49F-B74E-9F96-CE822D80671E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="22600" xr2:uid="{F0ABCEBB-BD47-304E-9491-7A7C2462A478}"/>
   </bookViews>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="469" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="468" uniqueCount="172">
   <si>
     <t>pair_id</t>
   </si>
@@ -1658,8 +1658,8 @@
       <c r="K15">
         <v>95</v>
       </c>
-      <c r="L15" s="1" t="s">
-        <v>20</v>
+      <c r="L15" s="1">
+        <v>1</v>
       </c>
       <c r="M15" s="1" t="s">
         <v>20</v>

</xml_diff>